<commit_message>
latest set of tables
</commit_message>
<xml_diff>
--- a/apcd_export_import/apcd_source_tables.xlsx
+++ b/apcd_export_import/apcd_source_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\temp\apcd\documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kc1-my.sharepoint.com/personal/jwhitehurst_kingcounty_gov/Documents/GitHub/claims_data/apcd_export_import/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174B367B-6618-4F55-8E8C-A82478677B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{174B367B-6618-4F55-8E8C-A82478677B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D422E5E1-D40F-420A-914F-710F7F309584}"/>
   <bookViews>
-    <workbookView xWindow="14235" yWindow="4755" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="93">
   <si>
     <t>schema_name</t>
   </si>
@@ -283,6 +283,27 @@
   </si>
   <si>
     <t>apcd_provider_master</t>
+  </si>
+  <si>
+    <t>final_apcd_elig_plr_2024</t>
+  </si>
+  <si>
+    <t>final_apcd_elig_month</t>
+  </si>
+  <si>
+    <t>ref_apcd_diagnosis_type</t>
+  </si>
+  <si>
+    <t>ref_apcd_drg_outlier_code</t>
+  </si>
+  <si>
+    <t>ref_apcd_medicare_termination_code</t>
+  </si>
+  <si>
+    <t>ref_apcd_race_code_imputed_external</t>
+  </si>
+  <si>
+    <t>ref_apcd_type_of_service</t>
   </si>
 </sst>
 </file>
@@ -600,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B82"/>
+  <dimension ref="A1:B89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -700,7 +721,7 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -708,7 +729,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -716,7 +737,7 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -724,7 +745,7 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -732,7 +753,7 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -740,7 +761,7 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -748,7 +769,7 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -756,7 +777,7 @@
         <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -764,7 +785,7 @@
         <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -772,7 +793,7 @@
         <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -780,7 +801,7 @@
         <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -788,7 +809,7 @@
         <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -796,7 +817,7 @@
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -804,7 +825,7 @@
         <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -812,7 +833,7 @@
         <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -820,7 +841,7 @@
         <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -828,7 +849,7 @@
         <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
@@ -836,7 +857,7 @@
         <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
@@ -844,7 +865,7 @@
         <v>2</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -852,7 +873,7 @@
         <v>2</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
@@ -860,7 +881,7 @@
         <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
@@ -868,7 +889,7 @@
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
@@ -876,7 +897,7 @@
         <v>2</v>
       </c>
       <c r="B34" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
@@ -884,7 +905,7 @@
         <v>2</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -892,7 +913,7 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -900,7 +921,7 @@
         <v>2</v>
       </c>
       <c r="B37" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -908,7 +929,7 @@
         <v>2</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>89</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -916,7 +937,7 @@
         <v>2</v>
       </c>
       <c r="B39" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -924,7 +945,7 @@
         <v>2</v>
       </c>
       <c r="B40" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
@@ -932,7 +953,7 @@
         <v>2</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -940,7 +961,7 @@
         <v>2</v>
       </c>
       <c r="B42" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -948,7 +969,7 @@
         <v>2</v>
       </c>
       <c r="B43" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
@@ -956,7 +977,7 @@
         <v>2</v>
       </c>
       <c r="B44" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
@@ -964,7 +985,7 @@
         <v>2</v>
       </c>
       <c r="B45" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
@@ -972,7 +993,7 @@
         <v>2</v>
       </c>
       <c r="B46" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
@@ -980,7 +1001,7 @@
         <v>2</v>
       </c>
       <c r="B47" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
@@ -988,7 +1009,7 @@
         <v>2</v>
       </c>
       <c r="B48" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
@@ -996,7 +1017,7 @@
         <v>2</v>
       </c>
       <c r="B49" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
@@ -1004,7 +1025,7 @@
         <v>2</v>
       </c>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
@@ -1012,7 +1033,7 @@
         <v>2</v>
       </c>
       <c r="B51" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
@@ -1020,7 +1041,7 @@
         <v>2</v>
       </c>
       <c r="B52" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
@@ -1028,7 +1049,7 @@
         <v>2</v>
       </c>
       <c r="B53" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
@@ -1036,7 +1057,7 @@
         <v>2</v>
       </c>
       <c r="B54" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
@@ -1044,7 +1065,7 @@
         <v>2</v>
       </c>
       <c r="B55" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
@@ -1052,7 +1073,7 @@
         <v>2</v>
       </c>
       <c r="B56" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
@@ -1060,7 +1081,7 @@
         <v>2</v>
       </c>
       <c r="B57" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
@@ -1068,7 +1089,7 @@
         <v>2</v>
       </c>
       <c r="B58" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
@@ -1076,7 +1097,7 @@
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
@@ -1084,7 +1105,7 @@
         <v>2</v>
       </c>
       <c r="B60" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
@@ -1092,7 +1113,7 @@
         <v>2</v>
       </c>
       <c r="B61" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
@@ -1100,7 +1121,7 @@
         <v>2</v>
       </c>
       <c r="B62" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
@@ -1108,7 +1129,7 @@
         <v>2</v>
       </c>
       <c r="B63" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
@@ -1116,7 +1137,7 @@
         <v>2</v>
       </c>
       <c r="B64" t="s">
-        <v>65</v>
+        <v>91</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -1124,7 +1145,7 @@
         <v>2</v>
       </c>
       <c r="B65" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -1132,7 +1153,7 @@
         <v>2</v>
       </c>
       <c r="B66" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
@@ -1140,7 +1161,7 @@
         <v>2</v>
       </c>
       <c r="B67" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -1148,7 +1169,7 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
@@ -1156,7 +1177,7 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -1164,7 +1185,7 @@
         <v>2</v>
       </c>
       <c r="B70" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
@@ -1172,7 +1193,7 @@
         <v>2</v>
       </c>
       <c r="B71" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
@@ -1180,7 +1201,7 @@
         <v>2</v>
       </c>
       <c r="B72" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
@@ -1188,78 +1209,134 @@
         <v>2</v>
       </c>
       <c r="B73" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="B74" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="B75" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="B76" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="B77" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="B78" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="B79" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="B80" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B81" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>75</v>
+      </c>
+      <c r="B82" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>78</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B83" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>78</v>
+      </c>
+      <c r="B84" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>78</v>
+      </c>
+      <c r="B85" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>78</v>
+      </c>
+      <c r="B86" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>78</v>
+      </c>
+      <c r="B87" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>78</v>
+      </c>
+      <c r="B88" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>78</v>
+      </c>
+      <c r="B89" t="s">
         <v>85</v>
       </c>
     </row>

</xml_diff>